<commit_message>
Minor changes due to excel saves.
</commit_message>
<xml_diff>
--- a/data/model-train-time-s-4.xlsx
+++ b/data/model-train-time-s-4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeffreylgoode/Documents/marketing-classifier-comparison/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CEF051D7-5045-B549-98CF-0EEEE0CB32EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3965F575-7940-8040-9FC6-ABE3D28311DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{C2313F39-8233-7346-AE10-D06809806728}"/>
   </bookViews>
@@ -386,7 +386,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -501,6 +501,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -546,10 +561,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -950,58 +966,58 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="3">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="3">
         <v>0.91</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="3">
         <v>0.91500000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="3">
         <v>0.15</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="3">
         <v>1</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="3">
         <v>0.88700000000000001</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="3">
         <v>3.2000000000000001E-2</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4" s="3">
         <v>0.92800000000000005</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3">
         <v>0.90500000000000003</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="3">
         <v>4.3719999999999999</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="3">
         <v>0.92200000000000004</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>0.91400000000000003</v>
       </c>
     </row>

</xml_diff>